<commit_message>
Email-first: read from the platform export, reach members by email
Skool's rules forbid bots and automated messages, so the skill never acts
inside the community platform. Members are read from the export and
reached from the owner's own email. On the call the owner says 'send it
now' or 'save it to my drafts'. The call opens with the whole picture
before any draft. New 'never_started' rule (joined, no intro or posts).
Opt-in voice notes over email quote the owner verbatim in Fo's voice.
Demo data gains email, posts and intro_posted columns.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WahaPgzRUVkS7qCQP8trx
</commit_message>
<xml_diff>
--- a/demo/coaching-skool/demo-member-sheet.xlsx
+++ b/demo/coaching-skool/demo-member-sheet.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q994"/>
+  <dimension ref="A1:T994"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="26" customWidth="1" style="18" min="1" max="1"/>
@@ -541,6 +541,21 @@
           <t>skip</t>
         </is>
       </c>
+      <c r="R1" s="19" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="S1" s="19" t="inlineStr">
+        <is>
+          <t>posts</t>
+        </is>
+      </c>
+      <c r="T1" s="19" t="inlineStr">
+        <is>
+          <t>intro_posted</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -589,6 +604,19 @@
       <c r="M2" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>owen.fontaine@example.com</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>29</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -637,6 +665,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>tomas.grimshaw@example.com</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>36</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -683,6 +724,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>terrence.vanderbilt@example.com</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>30</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -729,6 +783,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>niklas.voss@example.com</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>29</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -775,6 +842,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>quentin.wycliffe@example.com</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>33</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -821,6 +901,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>vernon.bramwell@example.com</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>38</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -867,6 +960,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>basil.whitfield@example.com</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>13</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -913,6 +1019,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>xavier.yates@example.com</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>12</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -965,6 +1084,19 @@
       <c r="M10" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>franklin.hawthorne@example.com</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>33</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1013,6 +1145,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>gavin.mumford@example.com</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>31</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1059,6 +1204,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>luigi.northgate@example.com</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>40</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1105,6 +1263,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>peter.sanderson@example.com</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>12</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1151,6 +1322,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>julius.yates@example.com</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>7</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1197,6 +1381,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>hamish.lindqvist@example.com</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>29</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="18">
       <c r="A16" s="9" t="inlineStr">
@@ -1243,6 +1440,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>silas.quigley@example.com</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>20</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="18">
       <c r="A17" s="9" t="inlineStr">
@@ -1289,6 +1499,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>padraig.fairbanks@example.com</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>10</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1337,6 +1560,19 @@
       <c r="M18" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>franklin.yarrow@example.com</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>6</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1385,6 +1621,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>stanley.pomeroy@example.com</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>35</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="18">
       <c r="A20" s="9" t="inlineStr">
@@ -1431,6 +1680,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>caleb.ashford@example.com</t>
+        </is>
+      </c>
+      <c r="S20" t="n">
+        <v>3</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="18">
       <c r="A21" s="9" t="inlineStr">
@@ -1477,6 +1739,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>derek.larimore@example.com</t>
+        </is>
+      </c>
+      <c r="S21" t="n">
+        <v>39</v>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="18">
       <c r="A22" s="9" t="inlineStr">
@@ -1523,6 +1798,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>enzo.ingram@example.com</t>
+        </is>
+      </c>
+      <c r="S22" t="n">
+        <v>26</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="18">
       <c r="A23" s="9" t="inlineStr">
@@ -1569,6 +1857,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>andrei.upton@example.com</t>
+        </is>
+      </c>
+      <c r="S23" t="n">
+        <v>29</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="18">
       <c r="A24" s="9" t="inlineStr">
@@ -1615,6 +1916,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>anders.zeigler@example.com</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>40</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="18">
       <c r="A25" s="9" t="inlineStr">
@@ -1663,6 +1977,19 @@
       <c r="M25" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>duncan.jamison@example.com</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>11</v>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -1711,6 +2038,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>karl.rowntree@example.com</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>40</v>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="18">
       <c r="A27" s="9" t="inlineStr">
@@ -1757,6 +2097,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>micah.yardley@example.com</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>1</v>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="18">
       <c r="A28" s="9" t="inlineStr">
@@ -1803,6 +2156,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>rafael.huxley@example.com</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>34</v>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="18">
       <c r="A29" s="9" t="inlineStr">
@@ -1849,6 +2215,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>xavier.jernigan@example.com</t>
+        </is>
+      </c>
+      <c r="S29" t="n">
+        <v>5</v>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="18">
       <c r="A30" s="9" t="inlineStr">
@@ -1895,6 +2274,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>luigi.winslow@example.com</t>
+        </is>
+      </c>
+      <c r="S30" t="n">
+        <v>4</v>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="18">
       <c r="A31" s="9" t="inlineStr">
@@ -1941,6 +2333,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>rowan.ridgeway@example.com</t>
+        </is>
+      </c>
+      <c r="S31" t="n">
+        <v>3</v>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="18">
       <c r="A32" s="9" t="inlineStr">
@@ -1987,6 +2392,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>silas.ingram@example.com</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>13</v>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="18">
       <c r="A33" s="9" t="inlineStr">
@@ -2033,6 +2451,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>lars.glendower@example.com</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>16</v>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="18">
       <c r="A34" s="9" t="inlineStr">
@@ -2081,6 +2512,19 @@
       <c r="M34" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>terrence.lachlan@example.com</t>
+        </is>
+      </c>
+      <c r="S34" t="n">
+        <v>39</v>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2129,6 +2573,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>ivan.montgomery@example.com</t>
+        </is>
+      </c>
+      <c r="S35" t="n">
+        <v>2</v>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="18">
       <c r="A36" s="9" t="inlineStr">
@@ -2175,6 +2632,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>xavier.ashford@example.com</t>
+        </is>
+      </c>
+      <c r="S36" t="n">
+        <v>30</v>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="18">
       <c r="A37" s="9" t="inlineStr">
@@ -2221,6 +2691,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>mateo.calloway@example.com</t>
+        </is>
+      </c>
+      <c r="S37" t="n">
+        <v>21</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="18">
       <c r="A38" s="9" t="inlineStr">
@@ -2267,6 +2750,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>peter.jamison@example.com</t>
+        </is>
+      </c>
+      <c r="S38" t="n">
+        <v>29</v>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="18">
       <c r="A39" s="9" t="inlineStr">
@@ -2313,6 +2809,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>levi.pruitt@example.com</t>
+        </is>
+      </c>
+      <c r="S39" t="n">
+        <v>38</v>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="18">
       <c r="A40" s="9" t="inlineStr">
@@ -2361,6 +2870,19 @@
       <c r="M40" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>padraig.fairview@example.com</t>
+        </is>
+      </c>
+      <c r="S40" t="n">
+        <v>13</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -2409,6 +2931,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>angus.quigley@example.com</t>
+        </is>
+      </c>
+      <c r="S41" t="n">
+        <v>34</v>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="18">
       <c r="A42" s="9" t="inlineStr">
@@ -2455,6 +2990,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>harold.tavish@example.com</t>
+        </is>
+      </c>
+      <c r="S42" t="n">
+        <v>15</v>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="18">
       <c r="A43" s="9" t="inlineStr">
@@ -2501,6 +3049,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>edmund.grimshaw@example.com</t>
+        </is>
+      </c>
+      <c r="S43" t="n">
+        <v>19</v>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="18">
       <c r="A44" s="9" t="inlineStr">
@@ -2547,6 +3108,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>callum.dunhill@example.com</t>
+        </is>
+      </c>
+      <c r="S44" t="n">
+        <v>32</v>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="18">
       <c r="A45" s="9" t="inlineStr">
@@ -2593,6 +3167,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>levi.yardley@example.com</t>
+        </is>
+      </c>
+      <c r="S45" t="n">
+        <v>1</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="18">
       <c r="A46" s="9" t="inlineStr">
@@ -2639,6 +3226,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>xavier.ingram@example.com</t>
+        </is>
+      </c>
+      <c r="S46" t="n">
+        <v>6</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="18">
       <c r="A47" s="9" t="inlineStr">
@@ -2685,6 +3285,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>nathaniel.quimby@example.com</t>
+        </is>
+      </c>
+      <c r="S47" t="n">
+        <v>30</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="18">
       <c r="A48" s="9" t="inlineStr">
@@ -2731,6 +3344,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>derek.sinclair@example.com</t>
+        </is>
+      </c>
+      <c r="S48" t="n">
+        <v>18</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="18">
       <c r="A49" s="9" t="inlineStr">
@@ -2777,6 +3403,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>andre.marlowe@example.com</t>
+        </is>
+      </c>
+      <c r="S49" t="n">
+        <v>27</v>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="18">
       <c r="A50" s="9" t="inlineStr">
@@ -2823,6 +3462,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>clifford.quimby@example.com</t>
+        </is>
+      </c>
+      <c r="S50" t="n">
+        <v>36</v>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="18">
       <c r="A51" s="9" t="inlineStr">
@@ -2869,6 +3521,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>clifford.eastwood@example.com</t>
+        </is>
+      </c>
+      <c r="S51" t="n">
+        <v>6</v>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="18">
       <c r="A52" s="9" t="inlineStr">
@@ -2915,6 +3580,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>angus.orchard@example.com</t>
+        </is>
+      </c>
+      <c r="S52" t="n">
+        <v>17</v>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="18">
       <c r="A53" s="9" t="inlineStr">
@@ -2961,6 +3639,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>stefan.fairview@example.com</t>
+        </is>
+      </c>
+      <c r="S53" t="n">
+        <v>21</v>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="18">
       <c r="A54" s="9" t="inlineStr">
@@ -3009,6 +3700,19 @@
       <c r="M54" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>malcolm.corbin@example.com</t>
+        </is>
+      </c>
+      <c r="S54" t="n">
+        <v>15</v>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -3057,6 +3761,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>oscar.fenwick@example.com</t>
+        </is>
+      </c>
+      <c r="S55" t="n">
+        <v>33</v>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="18">
       <c r="A56" s="9" t="inlineStr">
@@ -3103,6 +3820,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R56" t="inlineStr">
+        <is>
+          <t>adam.carmichael@example.com</t>
+        </is>
+      </c>
+      <c r="S56" t="n">
+        <v>19</v>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="18">
       <c r="A57" s="9" t="inlineStr">
@@ -3149,6 +3879,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R57" t="inlineStr">
+        <is>
+          <t>andrei.pruitt@example.com</t>
+        </is>
+      </c>
+      <c r="S57" t="n">
+        <v>2</v>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="18">
       <c r="A58" s="9" t="inlineStr">
@@ -3195,6 +3938,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R58" t="inlineStr">
+        <is>
+          <t>cedric.montgomery@example.com</t>
+        </is>
+      </c>
+      <c r="S58" t="n">
+        <v>0</v>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="18">
       <c r="A59" s="9" t="inlineStr">
@@ -3241,6 +3997,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>jonah.thornbury@example.com</t>
+        </is>
+      </c>
+      <c r="S59" t="n">
+        <v>26</v>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="18">
       <c r="A60" s="9" t="inlineStr">
@@ -3289,6 +4058,19 @@
       <c r="M60" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr">
+        <is>
+          <t>owen.yandell@example.com</t>
+        </is>
+      </c>
+      <c r="S60" t="n">
+        <v>0</v>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -3337,6 +4119,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R61" t="inlineStr">
+        <is>
+          <t>colin.zabriskie@example.com</t>
+        </is>
+      </c>
+      <c r="S61" t="n">
+        <v>5</v>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="18">
       <c r="A62" s="9" t="inlineStr">
@@ -3383,6 +4178,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>raymond.elbridge@example.com</t>
+        </is>
+      </c>
+      <c r="S62" t="n">
+        <v>1</v>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="18">
       <c r="A63" s="9" t="inlineStr">
@@ -3429,6 +4237,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>julian.northgate@example.com</t>
+        </is>
+      </c>
+      <c r="S63" t="n">
+        <v>0</v>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="18">
       <c r="A64" s="9" t="inlineStr">
@@ -3475,6 +4296,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>colin.thornbury@example.com</t>
+        </is>
+      </c>
+      <c r="S64" t="n">
+        <v>4</v>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="18">
       <c r="A65" s="9" t="inlineStr">
@@ -3521,6 +4355,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>inigo.corbin@example.com</t>
+        </is>
+      </c>
+      <c r="S65" t="n">
+        <v>31</v>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="18">
       <c r="A66" s="9" t="inlineStr">
@@ -3569,6 +4416,19 @@
       <c r="M66" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr">
+        <is>
+          <t>colin.winterbourne@example.com</t>
+        </is>
+      </c>
+      <c r="S66" t="n">
+        <v>26</v>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -3617,6 +4477,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>kendrick.kessler@example.com</t>
+        </is>
+      </c>
+      <c r="S67" t="n">
+        <v>37</v>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="18">
       <c r="A68" s="9" t="inlineStr">
@@ -3663,6 +4536,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>peter.thornbury@example.com</t>
+        </is>
+      </c>
+      <c r="S68" t="n">
+        <v>13</v>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="18">
       <c r="A69" s="9" t="inlineStr">
@@ -3709,6 +4595,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R69" t="inlineStr">
+        <is>
+          <t>emmett.wycliffe@example.com</t>
+        </is>
+      </c>
+      <c r="S69" t="n">
+        <v>18</v>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="18">
       <c r="A70" s="9" t="inlineStr">
@@ -3755,6 +4654,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>hugo.ridgeway@example.com</t>
+        </is>
+      </c>
+      <c r="S70" t="n">
+        <v>20</v>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="18">
       <c r="A71" s="9" t="inlineStr">
@@ -3801,6 +4713,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R71" t="inlineStr">
+        <is>
+          <t>levi.quimby@example.com</t>
+        </is>
+      </c>
+      <c r="S71" t="n">
+        <v>27</v>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="18">
       <c r="A72" s="9" t="inlineStr">
@@ -3847,6 +4772,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R72" t="inlineStr">
+        <is>
+          <t>hamish.oakeshott@example.com</t>
+        </is>
+      </c>
+      <c r="S72" t="n">
+        <v>8</v>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="18">
       <c r="A73" s="9" t="inlineStr">
@@ -3893,6 +4831,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R73" t="inlineStr">
+        <is>
+          <t>quentin.lindqvist@example.com</t>
+        </is>
+      </c>
+      <c r="S73" t="n">
+        <v>0</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="18">
       <c r="A74" s="9" t="inlineStr">
@@ -3941,6 +4892,19 @@
       <c r="M74" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr">
+        <is>
+          <t>wallace.pemberton@example.com</t>
+        </is>
+      </c>
+      <c r="S74" t="n">
+        <v>1</v>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -3989,6 +4953,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R75" t="inlineStr">
+        <is>
+          <t>xavier.garrick@example.com</t>
+        </is>
+      </c>
+      <c r="S75" t="n">
+        <v>0</v>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15.75" customHeight="1" s="18">
       <c r="A76" s="9" t="inlineStr">
@@ -4035,6 +5012,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>marco.mowbray@example.com</t>
+        </is>
+      </c>
+      <c r="S76" t="n">
+        <v>12</v>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="15.75" customHeight="1" s="18">
       <c r="A77" s="9" t="inlineStr">
@@ -4081,6 +5071,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>terrence.islington@example.com</t>
+        </is>
+      </c>
+      <c r="S77" t="n">
+        <v>13</v>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="18">
       <c r="A78" s="9" t="inlineStr">
@@ -4127,6 +5130,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R78" t="inlineStr">
+        <is>
+          <t>peter.fairview@example.com</t>
+        </is>
+      </c>
+      <c r="S78" t="n">
+        <v>13</v>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15.75" customHeight="1" s="18">
       <c r="A79" s="9" t="inlineStr">
@@ -4175,6 +5191,19 @@
       <c r="M79" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R79" t="inlineStr">
+        <is>
+          <t>enzo.pomeroy@example.com</t>
+        </is>
+      </c>
+      <c r="S79" t="n">
+        <v>9</v>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -4223,6 +5252,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R80" t="inlineStr">
+        <is>
+          <t>callum.norwood@example.com</t>
+        </is>
+      </c>
+      <c r="S80" t="n">
+        <v>25</v>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="18">
       <c r="A81" s="9" t="inlineStr">
@@ -4269,6 +5311,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R81" t="inlineStr">
+        <is>
+          <t>tomas.kirkland@example.com</t>
+        </is>
+      </c>
+      <c r="S81" t="n">
+        <v>0</v>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="18">
       <c r="A82" s="9" t="inlineStr">
@@ -4315,6 +5370,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R82" t="inlineStr">
+        <is>
+          <t>terrence.quimby@example.com</t>
+        </is>
+      </c>
+      <c r="S82" t="n">
+        <v>14</v>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="15.75" customHeight="1" s="18">
       <c r="A83" s="9" t="inlineStr">
@@ -4361,6 +5429,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>fraser.islington@example.com</t>
+        </is>
+      </c>
+      <c r="S83" t="n">
+        <v>0</v>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="18">
       <c r="A84" s="9" t="inlineStr">
@@ -4407,6 +5488,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R84" t="inlineStr">
+        <is>
+          <t>julian.quimby@example.com</t>
+        </is>
+      </c>
+      <c r="S84" t="n">
+        <v>38</v>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="15.75" customHeight="1" s="18">
       <c r="A85" s="9" t="inlineStr">
@@ -4455,6 +5549,19 @@
       <c r="M85" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R85" t="inlineStr">
+        <is>
+          <t>mateo.fairbanks@example.com</t>
+        </is>
+      </c>
+      <c r="S85" t="n">
+        <v>2</v>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -4503,6 +5610,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R86" t="inlineStr">
+        <is>
+          <t>fraser.sanderson@example.com</t>
+        </is>
+      </c>
+      <c r="S86" t="n">
+        <v>0</v>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="15.75" customHeight="1" s="18">
       <c r="A87" s="9" t="inlineStr">
@@ -4549,6 +5669,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R87" t="inlineStr">
+        <is>
+          <t>fraser.ironside@example.com</t>
+        </is>
+      </c>
+      <c r="S87" t="n">
+        <v>39</v>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="15.75" customHeight="1" s="18">
       <c r="A88" s="9" t="inlineStr">
@@ -4595,6 +5728,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R88" t="inlineStr">
+        <is>
+          <t>wallace.clayborne@example.com</t>
+        </is>
+      </c>
+      <c r="S88" t="n">
+        <v>37</v>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="18">
       <c r="A89" s="9" t="inlineStr">
@@ -4641,6 +5787,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>andre.zeigler@example.com</t>
+        </is>
+      </c>
+      <c r="S89" t="n">
+        <v>7</v>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="15.75" customHeight="1" s="18">
       <c r="A90" s="9" t="inlineStr">
@@ -4687,6 +5846,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>duncan.ironside@example.com</t>
+        </is>
+      </c>
+      <c r="S90" t="n">
+        <v>0</v>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="15.75" customHeight="1" s="18">
       <c r="A91" s="9" t="inlineStr">
@@ -4733,6 +5905,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>julian.waverly@example.com</t>
+        </is>
+      </c>
+      <c r="S91" t="n">
+        <v>0</v>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="15.75" customHeight="1" s="18">
       <c r="A92" s="9" t="inlineStr">
@@ -4779,6 +5964,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>silas.hawthorne@example.com</t>
+        </is>
+      </c>
+      <c r="S92" t="n">
+        <v>1</v>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="15.75" customHeight="1" s="18">
       <c r="A93" s="9" t="inlineStr">
@@ -4825,6 +6023,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>nathan.pemberton@example.com</t>
+        </is>
+      </c>
+      <c r="S93" t="n">
+        <v>22</v>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="15.75" customHeight="1" s="18">
       <c r="A94" s="9" t="inlineStr">
@@ -4871,6 +6082,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>paolo.sanderson@example.com</t>
+        </is>
+      </c>
+      <c r="S94" t="n">
+        <v>19</v>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="15.75" customHeight="1" s="18">
       <c r="A95" s="9" t="inlineStr">
@@ -4917,6 +6141,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>emmett.sinclair@example.com</t>
+        </is>
+      </c>
+      <c r="S95" t="n">
+        <v>5</v>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="15.75" customHeight="1" s="18">
       <c r="A96" s="9" t="inlineStr">
@@ -4963,6 +6200,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>clifford.cranfield@example.com</t>
+        </is>
+      </c>
+      <c r="S96" t="n">
+        <v>0</v>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="18">
       <c r="A97" s="9" t="inlineStr">
@@ -5009,6 +6259,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R97" t="inlineStr">
+        <is>
+          <t>marcus.radcliffe@example.com</t>
+        </is>
+      </c>
+      <c r="S97" t="n">
+        <v>16</v>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="18">
       <c r="A98" s="9" t="inlineStr">
@@ -5055,6 +6318,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R98" t="inlineStr">
+        <is>
+          <t>franklin.thornbury@example.com</t>
+        </is>
+      </c>
+      <c r="S98" t="n">
+        <v>0</v>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="15.75" customHeight="1" s="18">
       <c r="A99" s="9" t="inlineStr">
@@ -5101,6 +6377,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>leonard.whitfield@example.com</t>
+        </is>
+      </c>
+      <c r="S99" t="n">
+        <v>40</v>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="18">
       <c r="A100" s="9" t="inlineStr">
@@ -5147,6 +6436,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R100" t="inlineStr">
+        <is>
+          <t>rowan.jetley@example.com</t>
+        </is>
+      </c>
+      <c r="S100" t="n">
+        <v>38</v>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="18">
       <c r="A101" s="9" t="inlineStr">
@@ -5193,6 +6495,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R101" t="inlineStr">
+        <is>
+          <t>julius.jardine@example.com</t>
+        </is>
+      </c>
+      <c r="S101" t="n">
+        <v>37</v>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="102" ht="15.75" customHeight="1" s="18">
       <c r="A102" s="9" t="inlineStr">
@@ -5239,6 +6554,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R102" t="inlineStr">
+        <is>
+          <t>lars.underhill@example.com</t>
+        </is>
+      </c>
+      <c r="S102" t="n">
+        <v>0</v>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="103" ht="15.75" customHeight="1" s="18">
       <c r="A103" s="9" t="inlineStr">
@@ -5285,6 +6613,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R103" t="inlineStr">
+        <is>
+          <t>nathaniel.lachlan@example.com</t>
+        </is>
+      </c>
+      <c r="S103" t="n">
+        <v>10</v>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15.75" customHeight="1" s="18">
       <c r="A104" s="9" t="inlineStr">
@@ -5331,6 +6672,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R104" t="inlineStr">
+        <is>
+          <t>grant.ridgeway@example.com</t>
+        </is>
+      </c>
+      <c r="S104" t="n">
+        <v>15</v>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15.75" customHeight="1" s="18">
       <c r="A105" s="9" t="inlineStr">
@@ -5377,6 +6731,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R105" t="inlineStr">
+        <is>
+          <t>tomas.hollingsworth@example.com</t>
+        </is>
+      </c>
+      <c r="S105" t="n">
+        <v>40</v>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="106" ht="15.75" customHeight="1" s="18">
       <c r="A106" s="9" t="inlineStr">
@@ -5423,6 +6790,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R106" t="inlineStr">
+        <is>
+          <t>silas.fairview@example.com</t>
+        </is>
+      </c>
+      <c r="S106" t="n">
+        <v>13</v>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="107" ht="15.75" customHeight="1" s="18">
       <c r="A107" s="9" t="inlineStr">
@@ -5469,6 +6849,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R107" t="inlineStr">
+        <is>
+          <t>franklin.orchard@example.com</t>
+        </is>
+      </c>
+      <c r="S107" t="n">
+        <v>0</v>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="15.75" customHeight="1" s="18">
       <c r="A108" s="9" t="inlineStr">
@@ -5515,6 +6908,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>martin.lindqvist@example.com</t>
+        </is>
+      </c>
+      <c r="S108" t="n">
+        <v>36</v>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="109" ht="15.75" customHeight="1" s="18">
       <c r="A109" s="9" t="inlineStr">
@@ -5561,6 +6967,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R109" t="inlineStr">
+        <is>
+          <t>bruno.rothbury@example.com</t>
+        </is>
+      </c>
+      <c r="S109" t="n">
+        <v>0</v>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="15.75" customHeight="1" s="18">
       <c r="A110" s="9" t="inlineStr">
@@ -5607,6 +7026,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R110" t="inlineStr">
+        <is>
+          <t>callum.kelso@example.com</t>
+        </is>
+      </c>
+      <c r="S110" t="n">
+        <v>31</v>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="111" ht="15.75" customHeight="1" s="18">
       <c r="A111" s="9" t="inlineStr">
@@ -5653,6 +7085,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R111" t="inlineStr">
+        <is>
+          <t>emmett.trenchard@example.com</t>
+        </is>
+      </c>
+      <c r="S111" t="n">
+        <v>27</v>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15.75" customHeight="1" s="18">
       <c r="A112" s="9" t="inlineStr">
@@ -5699,6 +7144,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R112" t="inlineStr">
+        <is>
+          <t>mateo.yardley@example.com</t>
+        </is>
+      </c>
+      <c r="S112" t="n">
+        <v>0</v>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15.75" customHeight="1" s="18">
       <c r="A113" s="9" t="inlineStr">
@@ -5745,6 +7203,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R113" t="inlineStr">
+        <is>
+          <t>stanley.bramwell@example.com</t>
+        </is>
+      </c>
+      <c r="S113" t="n">
+        <v>0</v>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15.75" customHeight="1" s="18">
       <c r="A114" s="9" t="inlineStr">
@@ -5791,6 +7262,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R114" t="inlineStr">
+        <is>
+          <t>wallace.lindqvist@example.com</t>
+        </is>
+      </c>
+      <c r="S114" t="n">
+        <v>17</v>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15.75" customHeight="1" s="18">
       <c r="A115" s="9" t="inlineStr">
@@ -5837,6 +7321,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R115" t="inlineStr">
+        <is>
+          <t>paolo.ingram@example.com</t>
+        </is>
+      </c>
+      <c r="S115" t="n">
+        <v>26</v>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15.75" customHeight="1" s="18">
       <c r="A116" s="9" t="inlineStr">
@@ -5883,6 +7380,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R116" t="inlineStr">
+        <is>
+          <t>oscar.selwyn@example.com</t>
+        </is>
+      </c>
+      <c r="S116" t="n">
+        <v>39</v>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15.75" customHeight="1" s="18">
       <c r="A117" s="9" t="inlineStr">
@@ -5929,6 +7439,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R117" t="inlineStr">
+        <is>
+          <t>ivan.tavish@example.com</t>
+        </is>
+      </c>
+      <c r="S117" t="n">
+        <v>34</v>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="118" ht="15.75" customHeight="1" s="18">
       <c r="A118" s="9" t="inlineStr">
@@ -5975,6 +7498,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R118" t="inlineStr">
+        <is>
+          <t>declan.halewood@example.com</t>
+        </is>
+      </c>
+      <c r="S118" t="n">
+        <v>0</v>
+      </c>
+      <c r="T118" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="15.75" customHeight="1" s="18">
       <c r="A119" s="9" t="inlineStr">
@@ -6021,6 +7557,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R119" t="inlineStr">
+        <is>
+          <t>vernon.harrington@example.com</t>
+        </is>
+      </c>
+      <c r="S119" t="n">
+        <v>5</v>
+      </c>
+      <c r="T119" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="120" ht="15.75" customHeight="1" s="18">
       <c r="A120" s="9" t="inlineStr">
@@ -6067,6 +7616,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R120" t="inlineStr">
+        <is>
+          <t>leonard.rowntree@example.com</t>
+        </is>
+      </c>
+      <c r="S120" t="n">
+        <v>0</v>
+      </c>
+      <c r="T120" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="15.75" customHeight="1" s="18">
       <c r="A121" s="9" t="inlineStr">
@@ -6113,6 +7675,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R121" t="inlineStr">
+        <is>
+          <t>alvaro.montgomery@example.com</t>
+        </is>
+      </c>
+      <c r="S121" t="n">
+        <v>40</v>
+      </c>
+      <c r="T121" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="122" ht="15.75" customHeight="1" s="18">
       <c r="A122" s="9" t="inlineStr">
@@ -6159,6 +7734,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R122" t="inlineStr">
+        <is>
+          <t>tomas.upton@example.com</t>
+        </is>
+      </c>
+      <c r="S122" t="n">
+        <v>18</v>
+      </c>
+      <c r="T122" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="123" ht="15.75" customHeight="1" s="18">
       <c r="A123" s="9" t="inlineStr">
@@ -6205,6 +7793,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R123" t="inlineStr">
+        <is>
+          <t>ross.fairbanks@example.com</t>
+        </is>
+      </c>
+      <c r="S123" t="n">
+        <v>0</v>
+      </c>
+      <c r="T123" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="124" ht="15.75" customHeight="1" s="18">
       <c r="A124" s="9" t="inlineStr">
@@ -6251,6 +7852,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R124" t="inlineStr">
+        <is>
+          <t>jonah.radcliffe@example.com</t>
+        </is>
+      </c>
+      <c r="S124" t="n">
+        <v>2</v>
+      </c>
+      <c r="T124" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15.75" customHeight="1" s="18">
       <c r="A125" s="9" t="inlineStr">
@@ -6297,6 +7911,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R125" t="inlineStr">
+        <is>
+          <t>ivan.winterbourne@example.com</t>
+        </is>
+      </c>
+      <c r="S125" t="n">
+        <v>0</v>
+      </c>
+      <c r="T125" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15.75" customHeight="1" s="18">
       <c r="A126" s="9" t="inlineStr">
@@ -6343,6 +7970,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R126" t="inlineStr">
+        <is>
+          <t>diego.northgate@example.com</t>
+        </is>
+      </c>
+      <c r="S126" t="n">
+        <v>16</v>
+      </c>
+      <c r="T126" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="15.75" customHeight="1" s="18">
       <c r="A127" s="9" t="inlineStr">
@@ -6389,6 +8029,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R127" t="inlineStr">
+        <is>
+          <t>karl.ashcombe@example.com</t>
+        </is>
+      </c>
+      <c r="S127" t="n">
+        <v>0</v>
+      </c>
+      <c r="T127" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="128" ht="15.75" customHeight="1" s="18">
       <c r="A128" s="9" t="inlineStr">
@@ -6435,6 +8088,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R128" t="inlineStr">
+        <is>
+          <t>simon.pemberton@example.com</t>
+        </is>
+      </c>
+      <c r="S128" t="n">
+        <v>0</v>
+      </c>
+      <c r="T128" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="15.75" customHeight="1" s="18">
       <c r="A129" s="9" t="inlineStr">
@@ -6481,6 +8147,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R129" t="inlineStr">
+        <is>
+          <t>marcus.selwyn@example.com</t>
+        </is>
+      </c>
+      <c r="S129" t="n">
+        <v>37</v>
+      </c>
+      <c r="T129" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="15.75" customHeight="1" s="18">
       <c r="A130" s="9" t="inlineStr">
@@ -6527,6 +8206,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R130" t="inlineStr">
+        <is>
+          <t>martin.draper@example.com</t>
+        </is>
+      </c>
+      <c r="S130" t="n">
+        <v>6</v>
+      </c>
+      <c r="T130" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="15.75" customHeight="1" s="18">
       <c r="A131" s="9" t="inlineStr">
@@ -6573,6 +8265,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R131" t="inlineStr">
+        <is>
+          <t>raymond.jamison@example.com</t>
+        </is>
+      </c>
+      <c r="S131" t="n">
+        <v>29</v>
+      </c>
+      <c r="T131" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="132" ht="15.75" customHeight="1" s="18">
       <c r="A132" s="9" t="inlineStr">
@@ -6619,6 +8324,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R132" t="inlineStr">
+        <is>
+          <t>vernon.hollingsworth@example.com</t>
+        </is>
+      </c>
+      <c r="S132" t="n">
+        <v>34</v>
+      </c>
+      <c r="T132" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="15.75" customHeight="1" s="18">
       <c r="A133" s="9" t="inlineStr">
@@ -6665,6 +8383,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R133" t="inlineStr">
+        <is>
+          <t>caleb.pemberton@example.com</t>
+        </is>
+      </c>
+      <c r="S133" t="n">
+        <v>9</v>
+      </c>
+      <c r="T133" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="15.75" customHeight="1" s="18">
       <c r="A134" s="9" t="inlineStr">
@@ -6711,6 +8442,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R134" t="inlineStr">
+        <is>
+          <t>cedric.zeigler@example.com</t>
+        </is>
+      </c>
+      <c r="S134" t="n">
+        <v>2</v>
+      </c>
+      <c r="T134" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="15.75" customHeight="1" s="18">
       <c r="A135" s="9" t="inlineStr">
@@ -6757,6 +8501,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R135" t="inlineStr">
+        <is>
+          <t>hugo.clayborne@example.com</t>
+        </is>
+      </c>
+      <c r="S135" t="n">
+        <v>23</v>
+      </c>
+      <c r="T135" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="15.75" customHeight="1" s="18">
       <c r="A136" s="9" t="inlineStr">
@@ -6803,6 +8560,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R136" t="inlineStr">
+        <is>
+          <t>ulysses.hollingsworth@example.com</t>
+        </is>
+      </c>
+      <c r="S136" t="n">
+        <v>20</v>
+      </c>
+      <c r="T136" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="18">
       <c r="A137" s="9" t="inlineStr">
@@ -6849,6 +8619,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R137" t="inlineStr">
+        <is>
+          <t>wallace.pruitt@example.com</t>
+        </is>
+      </c>
+      <c r="S137" t="n">
+        <v>3</v>
+      </c>
+      <c r="T137" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="15.75" customHeight="1" s="18">
       <c r="A138" s="9" t="inlineStr">
@@ -6897,6 +8680,19 @@
       <c r="M138" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R138" t="inlineStr">
+        <is>
+          <t>andrei.upshaw@example.com</t>
+        </is>
+      </c>
+      <c r="S138" t="n">
+        <v>0</v>
+      </c>
+      <c r="T138" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -6945,6 +8741,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R139" t="inlineStr">
+        <is>
+          <t>gavin.ellsworth@example.com</t>
+        </is>
+      </c>
+      <c r="S139" t="n">
+        <v>31</v>
+      </c>
+      <c r="T139" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="15.75" customHeight="1" s="18">
       <c r="A140" s="9" t="inlineStr">
@@ -6991,6 +8800,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>caleb.islington@example.com</t>
+        </is>
+      </c>
+      <c r="S140" t="n">
+        <v>0</v>
+      </c>
+      <c r="T140" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="15.75" customHeight="1" s="18">
       <c r="A141" s="9" t="inlineStr">
@@ -7037,6 +8859,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R141" t="inlineStr">
+        <is>
+          <t>erik.ostrander@example.com</t>
+        </is>
+      </c>
+      <c r="S141" t="n">
+        <v>9</v>
+      </c>
+      <c r="T141" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="142" ht="15.75" customHeight="1" s="18">
       <c r="A142" s="9" t="inlineStr">
@@ -7083,6 +8918,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R142" t="inlineStr">
+        <is>
+          <t>luca.upton@example.com</t>
+        </is>
+      </c>
+      <c r="S142" t="n">
+        <v>5</v>
+      </c>
+      <c r="T142" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="15.75" customHeight="1" s="18">
       <c r="A143" s="9" t="inlineStr">
@@ -7129,6 +8977,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R143" t="inlineStr">
+        <is>
+          <t>ivan.hollowell@example.com</t>
+        </is>
+      </c>
+      <c r="S143" t="n">
+        <v>0</v>
+      </c>
+      <c r="T143" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="144" ht="15.75" customHeight="1" s="18">
       <c r="A144" s="9" t="inlineStr">
@@ -7175,6 +9036,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R144" t="inlineStr">
+        <is>
+          <t>archer.nesbitt@example.com</t>
+        </is>
+      </c>
+      <c r="S144" t="n">
+        <v>3</v>
+      </c>
+      <c r="T144" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="145" ht="15.75" customHeight="1" s="18">
       <c r="A145" s="9" t="inlineStr">
@@ -7221,6 +9095,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>henrik.harrington@example.com</t>
+        </is>
+      </c>
+      <c r="S145" t="n">
+        <v>9</v>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="15.75" customHeight="1" s="18">
       <c r="A146" s="9" t="inlineStr">
@@ -7267,6 +9154,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>quentin.stanton@example.com</t>
+        </is>
+      </c>
+      <c r="S146" t="n">
+        <v>22</v>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="147" ht="15.75" customHeight="1" s="18">
       <c r="A147" s="9" t="inlineStr">
@@ -7313,6 +9213,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>grant.grimshaw@example.com</t>
+        </is>
+      </c>
+      <c r="S147" t="n">
+        <v>23</v>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="15.75" customHeight="1" s="18">
       <c r="A148" s="9" t="inlineStr">
@@ -7359,6 +9272,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>harold.zabriskie@example.com</t>
+        </is>
+      </c>
+      <c r="S148" t="n">
+        <v>6</v>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="15.75" customHeight="1" s="18">
       <c r="A149" s="9" t="inlineStr">
@@ -7405,6 +9331,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>wallace.lockhart@example.com</t>
+        </is>
+      </c>
+      <c r="S149" t="n">
+        <v>31</v>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="15.75" customHeight="1" s="18">
       <c r="A150" s="9" t="inlineStr">
@@ -7451,6 +9390,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>callum.tavish@example.com</t>
+        </is>
+      </c>
+      <c r="S150" t="n">
+        <v>27</v>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="15.75" customHeight="1" s="18">
       <c r="A151" s="9" t="inlineStr">
@@ -7497,6 +9449,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>hamish.dunhill@example.com</t>
+        </is>
+      </c>
+      <c r="S151" t="n">
+        <v>2</v>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="15.75" customHeight="1" s="18">
       <c r="A152" s="9" t="inlineStr">
@@ -7545,6 +9510,19 @@
       <c r="M152" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>luigi.osborne@example.com</t>
+        </is>
+      </c>
+      <c r="S152" t="n">
+        <v>32</v>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
     </row>
@@ -7593,6 +9571,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>nathan.lindqvist@example.com</t>
+        </is>
+      </c>
+      <c r="S153" t="n">
+        <v>37</v>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="15.75" customHeight="1" s="18">
       <c r="A154" s="8" t="inlineStr">
@@ -7636,6 +9627,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>mateo.fenwick@example.com</t>
+        </is>
+      </c>
+      <c r="S154" t="n">
+        <v>0</v>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="15.75" customHeight="1" s="18">
       <c r="A155" s="8" t="inlineStr">
@@ -7679,6 +9683,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>simon.yarrow@example.com</t>
+        </is>
+      </c>
+      <c r="S155" t="n">
+        <v>25</v>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="15.75" customHeight="1" s="18">
       <c r="A156" s="8" t="inlineStr">
@@ -7722,6 +9739,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>milan.upshaw@example.com</t>
+        </is>
+      </c>
+      <c r="S156" t="n">
+        <v>39</v>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="15.75" customHeight="1" s="18">
       <c r="A157" s="8" t="inlineStr">
@@ -7763,6 +9793,19 @@
       <c r="M157" s="0" t="inlineStr">
         <is>
           <t>none</t>
+        </is>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>terrence.prescott@example.com</t>
+        </is>
+      </c>
+      <c r="S157" t="n">
+        <v>0</v>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -7784,6 +9827,19 @@
           <t>none</t>
         </is>
       </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>nathaniel.pomeroy@example.com</t>
+        </is>
+      </c>
+      <c r="S158" t="n">
+        <v>6</v>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="15.75" customHeight="1" s="18">
       <c r="A159" s="0" t="inlineStr">
@@ -7840,6 +9896,14 @@
       <c r="N159" s="0" t="inlineStr">
         <is>
           <t>&lt;your profile link in the test community&gt;</t>
+        </is>
+      </c>
+      <c r="S159" t="n">
+        <v>0</v>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
@@ -20071,7 +22135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="130" customWidth="1" style="18" min="1" max="1"/>
@@ -20140,7 +22204,7 @@
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>channel: 'none' = draft and review only, never sent. During setup, Fo fills in the tester row(s) with a real name and profile link and sets channel to 'skool'; only those rows can receive a real message.</t>
+          <t>channel: 'none' = draft and review only, never sent. During setup, Fo fills in the tester row(s) with a real name and email and sets channel to 'email'; only those rows can receive a real message.</t>
         </is>
       </c>
     </row>
@@ -20162,6 +22226,13 @@
       <c r="A13" s="0" t="inlineStr">
         <is>
           <t>Status history, Drafts, Conversions, Checks, Scorecard and Run log are written by Fo and Claude. Don't edit them by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>email, posts, intro_posted: from the member export. Emails here are fictional (example.com). posts = 0 and intro_posted = no means the member never got started.</t>
         </is>
       </c>
     </row>

</xml_diff>